<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-05 Le bateau d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-05.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre, cuisine, jardin, le matin</t>
+          <t>chambre, cuisine, jardin, arrosoir sur le bassin, le matin</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire flotter sa noix dans le bassin. Il part en pyjama, le bassin est vide. Une chose puis la suivante, la feuille-voile avance sur l'eau.</t>
+          <t>Dans le jardin, l'arrosoir tape le bassin vide. Sur la noix, un éclat de quille luit. Amir veut flotter maintenant. Il prend tout : la feuille s'envole, la noix glisse, l'éclat disparaît. Papa s'accroupit. Merci vécu. Il refuse de foncer. Sur l'eau, l'éclat de quille reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur la table de nuit, une noix attend. À côté, une petite feuille sèche. La feuille est légère, presque rien. La noix a un dos tout ridé. Un rayon jaune allonge deux pantoufles. On dirait deux petits quais. La poussière danse dans le rayon. Amir, tu vois ta noix ? Oui, papa. C'est le bateau. Le bassin est dans le jardin. En ce moment, Amir ouvre les yeux. Il prend la noix tout de suite. Il glisse les pieds dans les pantoufles. On va à l'eau. Il marche vers la porte, encore en pyjama. Le bassin, dehors, est encore vide. L'eau arrive, tout doucement. Et nous aussi. Une chose, puis la suivante. Amir s'arrête sur le tapis crème. La noix est chaude dans sa main. Elle veut flotter. Elle flottera. D'abord on s'habille. On se lève pour de bon ? Oui. Amir repose la noix près de la feuille. Le rayon touche encore les pantoufles. Le pull rouge, sur le dossier.</t>
+          <t>Dans le jardin, l'arrosoir tape le bassin. Le métal est froid, un peu creux. Dans la chambre, une feuille sèche cliquette. Elle est posée près d'une noix ridée. Un éclat de quille luit sur son dos. Il brille, papa. Tu le vois, sur le bois de la noix ? Deux pantoufles allongent des quais jaunes. Un rayon les touche, près du tapis crème. La poussière danse dans le rayon. Le bassin du jardin attend de l'eau. L'air sent la banane, depuis la cuisine. J'ai coupé un fruit, Amir. Mon bateau va flotter, maintenant ! Ta noix veut l'eau, Amir. En ce moment, Amir saisit noix et feuille. Il glisse les pieds dans les pantoufles. Il marche vers la porte, en pyjama. On va à l'eau ! La feuille s'envole derrière la chaise. La noix bascule, et l'éclat de quille disparaît. Oh ! Le sourire d'Amir disparaît. Dehors, le bassin est vide, gris. Il n'y a pas d'eau. L'eau n'est pas versée. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends tout, et j'y vais ! Il ramasse noix, feuille, pantoufles d'un coup. La noix glisse, clac, sous le lit. L'éclat de quille s'est caché. Il est perdu.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur la table de nuit, une noix attend. À côté, une petite feuille sèche. La feuille est légère, presque rien. La noix a un dos tout ridé. Un rayon jaune allonge deux pantoufles. On dirait deux petits quais. La poussière danse dans le rayon. Amir, tu vois ta noix ? Oui, papa. C'est le bateau. Le bassin est dans le jardin. En ce moment, Amir ouvre les yeux. Il prend la noix tout de suite. Il glisse les pieds dans les pantoufles. On va à l'eau. Il marche vers la porte, encore en pyjama. Le bassin, dehors, est encore vide. L'eau arrive, tout doucement. Et nous aussi. Une chose, puis la suivante. Amir s'arrête sur le tapis crème. La noix est chaude dans sa main. Elle veut flotter. Elle flottera. D'abord on s'habille. On se lève pour de bon ? Oui. Amir repose la noix près de la feuille. Le rayon touche encore les pantoufles. Le pull rouge, sur le dossier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans le jardin, l'arrosoir tape le bassin. Le métal est froid, un peu creux. Dans la chambre, une feuille sèche cliquette. Elle est posée près d'une noix ridée. Un &lt;emphasis level="moderate"&gt;éclat de quille&lt;/emphasis&gt; luit sur son dos. Il brille, papa. Tu le vois, sur le bois de la noix ? Deux pantoufles allongent des quais jaunes. Un rayon les touche, près du tapis crème. La poussière danse dans le rayon. Le bassin du jardin attend de l'eau. L'air sent la banane, depuis la cuisine. J'ai coupé un fruit, Amir. Mon bateau va flotter, maintenant ! Ta noix veut l'eau, Amir. En ce moment, Amir saisit noix et feuille. Il glisse les pieds dans les pantoufles. Il marche vers la porte, en pyjama. On va à l'eau ! La feuille s'envole derrière la chaise. La noix bascule, et l'éclat de quille disparaît. Oh ! Le sourire d'Amir disparaît. Dehors, le bassin est vide, gris. Il n'y a pas d'eau. L'eau n'est pas versée. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends tout, et j'y vais ! Il ramasse noix, feuille, pantoufles d'un coup. La noix glisse, clac, sous le lit. L'éclat de quille s'est caché. Il est perdu.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil entre dans la chambre. Joséphine ouvre les yeux. Le drap est chaud. Maman dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Joséphine se lève. Ses pieds touchent le tapis. Ensuite, Joséphine s'habille. Elle met le pull vert. Elle met le pantalon. Les chaussettes aussi. Papa dit : maintenant, le déjeuner. Joséphine s'assoit à table. Elle mange du pain. Elle boit du lait tiède. Maman dit : ensuite, le sac. Joséphine met la gourde dans le sac. Elle met le cahier dans le sac. Chaque étape est finie, alors Joséphine est prête. Le lendemain, c'est samedi. Joséphine se souvient. Une étape après l'autre. Elle se lève. Elle s'habille. Elle déjeune. Elle prépare le petit sac pour le marché. Papa dit : tu as refait les étapes. Lever, habiller, déjeuner, sac. Joséphine sourit. C'est plus calme. [pause]</t>
+          <t>Dans le jardin, l'arrosoir tape le bassin. Le métal est froid, un peu creux. Dans la chambre, une feuille sèche cliquette. Elle est posée près d'une noix ridée. Un &lt;emphasis&gt;éclat de quille&lt;/emphasis&gt; luit sur son dos. Il brille, papa. Tu le vois, sur le bois de la noix ? Deux pantoufles allongent des quais jaunes. Un rayon les touche, près du tapis crème. La poussière danse dans le rayon. Le bassin du jardin attend de l'eau. L'air sent la banane, depuis la cuisine. J'ai coupé un fruit, Amir. Mon bateau va flotter, maintenant ! Ta noix veut l'eau, Amir. En ce moment, Amir saisit noix et feuille. Il glisse les pieds dans les pantoufles. Il marche vers la porte, en pyjama. On va à l'eau ! La feuille s'envole derrière la chaise. La noix bascule, et l'éclat de quille disparaît. Oh ! Le sourire d'Amir disparaît. Dehors, le bassin est vide, gris. Il n'y a pas d'eau. L'eau n'est pas versée. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends tout, et j'y vais ! Il ramasse noix, feuille, pantoufles d'un coup. La noix glisse, clac, sous le lit. L'éclat de quille s'est caché. Il est perdu. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de quille</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,44 +1321,50 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_noix_sur_l_eau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur la table de nuit, une noix attend.
-narrateur|À côté, une petite feuille sèche.
-narrateur|La feuille est légère, presque rien.
-narrateur|La noix a un dos tout ridé.
-narrateur|Un rayon jaune allonge deux pantoufles.
-narrateur|On dirait deux petits quais.
+          <t>narrateur|Dans le jardin, l'arrosoir tape le bassin.
+narrateur|Le métal est froid, un peu creux.
+narrateur|Dans la chambre, une feuille sèche cliquette.
+narrateur|Elle est posée près d'une noix ridée.
+narrateur|Un éclat de quille luit sur son dos.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le bois de la noix ?
+narrateur|Deux pantoufles allongent des quais jaunes.
+narrateur|Un rayon les touche, près du tapis crème.
 narrateur|La poussière danse dans le rayon.
-papa|Amir, tu vois ta noix ?
-enfant-m|Oui, papa.
-enfant-m|C'est le bateau.
-maman|Le bassin est dans le jardin.
-narrateur|En ce moment, Amir ouvre les yeux.
-narrateur|Il prend la noix tout de suite.
+maman|Le bassin du jardin attend de l'eau.
+narrateur|L'air sent la banane, depuis la cuisine.
+maman|J'ai coupé un fruit, Amir.
+enfant-m|Mon bateau va flotter, maintenant !
+papa|Ta noix veut l'eau, Amir.
+narrateur|En ce moment, Amir saisit noix et feuille.
 narrateur|Il glisse les pieds dans les pantoufles.
-enfant-m|On va à l'eau.
-narrateur|Il marche vers la porte, encore en pyjama.
-narrateur|Le bassin, dehors, est encore vide.
-papa|L'eau arrive, tout doucement.
-papa|Et nous aussi.
-maman|Une chose, puis la suivante.
-narrateur|Amir s'arrête sur le tapis crème.
-narrateur|La noix est chaude dans sa main.
-enfant-m|Elle veut flotter.
-maman|Elle flottera.
-maman|D'abord on s'habille.
-papa|On se lève pour de bon ?
-enfant-m|Oui.
-narrateur|Amir repose la noix près de la feuille.
-narrateur|Le rayon touche encore les pantoufles.
-papa|Le pull rouge, sur le dossier.</t>
+narrateur|Il marche vers la porte, en pyjama.
+enfant-m|On va à l'eau !
+narrateur|La feuille s'envole derrière la chaise.
+narrateur|La noix bascule, et l'éclat de quille disparaît.
+enfant-m|Oh !
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dehors, le bassin est vide, gris.
+enfant-m|Il n'y a pas d'eau.
+papa|L'eau n'est pas versée.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Je prends tout, et j'y vais !
+narrateur|Il ramasse noix, feuille, pantoufles d'un coup.
+narrateur|La noix glisse, clac, sous le lit.
+narrateur|L'éclat de quille s'est caché.
+enfant-m|Il est perdu.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>rayon</t>
+          <t>rayon,arrosoir</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1396,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir veut le bassin. Comment se prépare-t-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir veut le &lt;emphasis level="moderate"&gt;bassin&lt;/emphasis&gt;. Comment se prépare-t-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Joséphine se prépare. Comment avance-t-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir veut le &lt;emphasis&gt;bassin&lt;/emphasis&gt;. Comment se prépare-t-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1458,7 +1464,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1466,10 +1472,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,34 +1490,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>bassin</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1520,23 +1530,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_se_prepare_une_chose_apres_l_autre; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1569,17 +1579,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le pull. Le pull est un peu rêche aux poignets. Je suis habillé. La cuisine, maintenant. Ça sent la banane et le lait tiède. Tu veux la banane coupée ? Oui, maman. Amir s'assoit à table. La banane est douce, un peu sucrée. Dehors, je verse l'eau. Tu finis ton bol, et l'eau sera prête. D'accord. Il boit une gorgée de lait. Le lait est tiède contre la lèvre. Merci, Amir. Ensuite, le sac.</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes bien sous le lit ? Oui, papa. Amir pose la feuille sur la table. Puis il cherche, une main, près du tapis. Ses doigts trouvent la noix froide. Ma noix ! Un éclat de quille reparaît, pâle. Merci, tu l'as trouvée. Elle était dessous. Le pull rouge, sur le dossier. Amir enfile le pull. Le pull est rêche aux poignets. Je suis habillé. La cuisine, maintenant. Ça sent la banane et le lait tiède. Tu veux la banane coupée ? Oui, maman. Amir s'assoit à table. La banane est douce, un peu sucrée. Dehors, je verse l'eau. Tu finis ton bol, et l'eau sera prête. D'accord. Il boit une gorgée de lait. Le lait est tiède contre la lèvre. Ensuite, le sac.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir enfile le pull. Le pull est un peu rêche aux poignets. Je suis habillé. La cuisine, maintenant. Ça sent la banane et le lait tiède. Tu veux la banane coupée ? Oui, maman. Amir s'assoit à table. La banane est douce, un peu sucrée. Dehors, je verse l'eau. Tu finis ton bol, et l'eau sera prête. D'accord. Il boit une gorgée de lait. Le lait est tiède contre la lèvre. Merci, Amir. Ensuite, le sac.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Tu regardes bien sous le lit ? Oui, papa. Amir pose la feuille sur la table. Puis il cherche, une main, près du tapis. Ses doigts trouvent la noix froide. Ma noix ! Un &lt;emphasis level="moderate"&gt;éclat de quille&lt;/emphasis&gt; reparaît, pâle. Merci, tu l'as trouvée. Elle était dessous. Le pull rouge, sur le dossier. Amir enfile le pull. Le pull est rêche aux poignets. Je suis habillé. La cuisine, maintenant. Ça sent la banane et le lait tiède. Tu veux la banane coupée ? Oui, maman. Amir s'assoit à table. La banane est douce, un peu sucrée. Dehors, je verse l'eau. Tu finis ton bol, et l'eau sera prête. D'accord. Il boit une gorgée de lait. Le lait est tiède contre la lèvre. Ensuite, le sac.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Joséphine a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes bien sous le lit ? Oui, papa. Amir pose la feuille sur la table. Puis il cherche, une main, près du tapis. Ses doigts trouvent la noix froide. Ma noix ! Un &lt;emphasis&gt;éclat de quille&lt;/emphasis&gt; reparaît, pâle. Merci, tu l'as trouvée. Elle était dessous. Le pull rouge, sur le dossier. Amir enfile le pull. Le pull est rêche aux poignets. Je suis habillé. La cuisine, maintenant. Ça sent la banane et le lait tiède. Tu veux la banane coupée ? Oui, maman. Amir s'assoit à table. La banane est douce, un peu sucrée. Dehors, je verse l'eau. Tu finis ton bol, et l'eau sera prête. D'accord. Il boit une gorgée de lait. Le lait est tiède contre la lèvre. Ensuite, le sac. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1626,7 +1636,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1634,10 +1644,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1660,7 +1670,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de quille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1674,16 +1684,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1692,10 +1702,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1708,13 +1718,24 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_feuille_d_abord_puis_la_noix_sous_le_lit; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir enfile le pull.
-narrateur|Le pull est un peu rêche aux poignets.
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu regardes bien sous le lit ?
+enfant-m|Oui, papa.
+narrateur|Amir pose la feuille sur la table.
+narrateur|Puis il cherche, une main, près du tapis.
+narrateur|Ses doigts trouvent la noix froide.
+enfant-m|Ma noix !
+narrateur|Un éclat de quille reparaît, pâle.
+papa|Merci, tu l'as trouvée.
+enfant-m|Elle était dessous.
+maman|Le pull rouge, sur le dossier.
+narrateur|Amir enfile le pull.
+narrateur|Le pull est rêche aux poignets.
 enfant-m|Je suis habillé.
 maman|La cuisine, maintenant.
 narrateur|Ça sent la banane et le lait tiède.
@@ -1727,8 +1748,12 @@
 enfant-m|D'accord.
 narrateur|Il boit une gorgée de lait.
 narrateur|Le lait est tiède contre la lèvre.
-maman|Merci, Amir.
 maman|Ensuite, le sac.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>banane,lait</t>
         </is>
       </c>
     </row>
@@ -1755,17 +1780,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir met la gourde dans le sac. Il met le cahier. Il met la noix, tout au-dessus. La petite feuille aussi. Tu as mis le bateau ? Oui, papa. Amir range les pantoufles près du tapis. Tu les as remises au quai ? Oui. Maman ouvre la porte. L'air sent le jardin, un peu humide. Le bassin a un peu d'eau, toute calme. Amir pose la noix. Il pose la feuille dessus. Souffle, papa. Papa souffle. La noix avance, tout doucement. Elle flotte. Un petit rond d'eau s'ouvre. Encore, papa. Papa souffle encore, plus fort. La feuille-voile tremble, puis repart.</t>
+          <t>Amir met la gourde dans le sac. Il glisse le cahier à côté. Il pose la noix tout au-dessus. La feuille aussi. Tu as mis le bateau ? Oui, papa. Amir range les pantoufles près du tapis. Tu les as remises au quai ? Oui. Maman ouvre la porte. L'air sent le jardin, un peu humide. Le bassin a un peu d'eau, grise. Je jette tout, maintenant ! Il avance les mains vers le sac. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Amir observe la noix, écoute le jardin. Sur le dos, l'éclat de quille luit. Là, près de l'éclat. Il pose d'abord les pantoufles au bord. Deux petits quais, comme dans la chambre. Puis la noix, au creux de l'eau. La feuille-voile, maintenant. Tu souffles, ou je souffle ? Toi, papa. Papa souffle. La noix avance, lente, sur l'eau. Elle flotte. Un petit rond d'eau s'ouvre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir met la gourde dans le sac. Il met le cahier. Il met la noix, tout au-dessus. La petite feuille aussi. Tu as mis le bateau ? Oui, papa. Amir range les pantoufles près du tapis. Tu les as remises au quai ? Oui. Maman ouvre la porte. L'air sent le jardin, un peu humide. Le bassin a un peu d'eau, toute calme. Amir pose la noix. Il pose la feuille dessus. Souffle, papa. Papa souffle. La noix avance, tout doucement. Elle flotte. Un petit rond d'eau s'ouvre. Encore, papa. Papa souffle encore, plus fort. La feuille-voile tremble, puis repart.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir met la gourde dans le sac. Il glisse le cahier à côté. Il pose la noix tout au-dessus. La feuille aussi. Tu as mis le bateau ? Oui, papa. Amir range les pantoufles près du tapis. Tu les as remises au quai ? Oui. Maman ouvre la porte. L'air sent le jardin, un peu humide. Le bassin a un peu d'eau, grise. Je jette tout, maintenant ! Il avance les mains vers le sac. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Amir observe la noix, écoute le jardin. Sur le dos, l'&lt;emphasis level="moderate"&gt;éclat de quille&lt;/emphasis&gt; luit. Là, près de l'éclat. Il pose d'abord les pantoufles au bord. Deux petits quais, comme dans la chambre. Puis la noix, au creux de l'eau. La feuille-voile, maintenant. Tu souffles, ou je souffle ? Toi, papa. Papa souffle. La noix avance, lente, sur l'eau. Elle flotte. Un petit rond d'eau s'ouvre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Joséphine met les chaussures. Maman ouvre la porte. L'air sent le matin. [pause]</t>
+          <t>Amir met la gourde dans le sac. Il glisse le cahier à côté. Il pose la noix tout au-dessus. La feuille aussi. Tu as mis le bateau ? Oui, papa. Amir range les pantoufles près du tapis. Tu les as remises au quai ? Oui. Maman ouvre la porte. L'air sent le jardin, un peu humide. Le bassin a un peu d'eau, grise. Je jette tout, maintenant ! Il avance les mains vers le sac. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Amir observe la noix, écoute le jardin. Sur le dos, l'&lt;emphasis&gt;éclat de quille&lt;/emphasis&gt; luit. Là, près de l'éclat. Il pose d'abord les pantoufles au bord. Deux petits quais, comme dans la chambre. Puis la noix, au creux de l'eau. La feuille-voile, maintenant. Tu souffles, ou je souffle ? Toi, papa. Papa souffle. La noix avance, lente, sur l'eau. Elle flotte. Un petit rond d'eau s'ouvre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1812,7 +1837,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1820,10 +1845,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1844,28 +1869,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de quille</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1874,10 +1903,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1888,13 +1917,17 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Amir met la gourde dans le sac.
-narrateur|Il met le cahier.
-narrateur|Il met la noix, tout au-dessus.
-narrateur|La petite feuille aussi.
+narrateur|Il glisse le cahier à côté.
+narrateur|Il pose la noix tout au-dessus.
+enfant-m|La feuille aussi.
 papa|Tu as mis le bateau ?
 enfant-m|Oui, papa.
 narrateur|Amir range les pantoufles près du tapis.
@@ -1902,17 +1935,26 @@
 enfant-m|Oui.
 narrateur|Maman ouvre la porte.
 narrateur|L'air sent le jardin, un peu humide.
-narrateur|Le bassin a un peu d'eau, toute calme.
-narrateur|Amir pose la noix.
-narrateur|Il pose la feuille dessus.
-enfant-m|Souffle, papa.
+narrateur|Le bassin a un peu d'eau, grise.
+enfant-m|Je jette tout, maintenant !
+narrateur|Il avance les mains vers le sac.
+narrateur|Puis il s'arrête net.
+narrateur|Il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Amir observe la noix, écoute le jardin.
+narrateur|Sur le dos, l'éclat de quille luit.
+enfant-m|Là, près de l'éclat.
+narrateur|Il pose d'abord les pantoufles au bord.
+narrateur|Deux petits quais, comme dans la chambre.
+narrateur|Puis la noix, au creux de l'eau.
+enfant-m|La feuille-voile, maintenant.
+papa|Tu souffles, ou je souffle ?
+enfant-m|Toi, papa.
 narrateur|Papa souffle.
-narrateur|La noix avance, tout doucement.
+narrateur|La noix avance, lente, sur l'eau.
 maman|Elle flotte.
-narrateur|Un petit rond d'eau s'ouvre.
-enfant-m|Encore, papa.
-narrateur|Papa souffle encore, plus fort.
-narrateur|La feuille-voile tremble, puis repart.</t>
+narrateur|Un petit rond d'eau s'ouvre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1944,17 +1986,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est parti. Une chose, puis la suivante. Les pantoufles ont attendu, et toi tu as avancé. Le rayon revient sur le tapis, là-bas. Bravo, Amir. La noix glisse encore, toute petite, sur l'eau calme.</t>
+          <t>Le bateau est parti. Maman s'assoit au bord du bassin. Tu veux un bout de banane ? Oui, papa. La banane sent fort, sucrée. La noix a un petit éclat. Un éclat de quille tient sur l'eau. Tu le vois, comme sur la table ? Oui, maman. L'arrosoir se tait, dehors. Sur l'eau, l'éclat de quille reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau est parti. Une chose, puis la suivante. Les pantoufles ont attendu, et toi tu as avancé. Le rayon revient sur le tapis, là-bas. Bravo, Amir. La noix glisse encore, toute petite, sur l'eau calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le bateau est parti. Maman s'assoit au bord du bassin. Tu veux un bout de banane ? Oui, papa. La banane sent fort, sucrée. La noix a un petit éclat. Un &lt;emphasis level="moderate"&gt;éclat de quille&lt;/emphasis&gt; tient sur l'eau. Tu le vois, comme sur la table ? Oui, maman. L'arrosoir se tait, dehors. Sur l'eau, l'éclat de quille reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le bateau est parti. Maman s'assoit au bord du bassin. Tu veux un bout de banane ? Oui, papa. La banane sent fort, sucrée. La noix a un petit éclat. Un &lt;emphasis&gt;éclat de quille&lt;/emphasis&gt; tient sur l'eau. Tu le vois, comme sur la table ? Oui, maman. L'arrosoir se tait, dehors. Sur l'eau, l'éclat de quille reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2001,18 +2043,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2021,12 +2063,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2035,17 +2077,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de quille</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2054,11 +2100,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2067,29 +2113,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_eau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-m|Le bateau est parti.
-papa|Une chose, puis la suivante.
-maman|Les pantoufles ont attendu, et toi tu as avancé.
-narrateur|Le rayon revient sur le tapis, là-bas.
-papa|Bravo, Amir.
-narrateur|La noix glisse encore, toute petite, sur l'eau calme.</t>
+narrateur|Maman s'assoit au bord du bassin.
+papa|Tu veux un bout de banane ?
+enfant-m|Oui, papa.
+narrateur|La banane sent fort, sucrée.
+enfant-m|La noix a un petit éclat.
+narrateur|Un éclat de quille tient sur l'eau.
+maman|Tu le vois, comme sur la table ?
+enfant-m|Oui, maman.
+narrateur|L'arrosoir se tait, dehors.
+narrateur|Sur l'eau, l'éclat de quille reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>eau</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2202,6 +2262,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>